<commit_message>
Completion: Navigation to Open Task and JSON based flow
</commit_message>
<xml_diff>
--- a/testdata/payment_terms.xlsx
+++ b/testdata/payment_terms.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sriya\axiom\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{15C1E917-AC33-46D7-B8C4-741230C9CA40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6ADE1E9-46DE-4199-BFF2-40EC5842BAED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B9CEA518-74DE-486F-B3BF-39C5E59AD1FA}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="PaymentTerms" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,19 +40,19 @@
     <t>Action</t>
   </si>
   <si>
-    <t>TermName</t>
-  </si>
-  <si>
     <t>Description</t>
   </si>
   <si>
-    <t>DueDays</t>
-  </si>
-  <si>
     <t>CREATE</t>
   </si>
   <si>
     <t>Net 30 Demo</t>
+  </si>
+  <si>
+    <t>Term Name</t>
+  </si>
+  <si>
+    <t>Due Days</t>
   </si>
 </sst>
 </file>
@@ -414,7 +415,7 @@
   <cols>
     <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -422,24 +423,24 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D2" s="1">
         <v>30</v>

</xml_diff>